<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-07 La craie d'Amir
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-07.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-07.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>pas de la porte, platane du village, pierre du soir</t>
+          <t>école puis maison, pas de la porte, platane du village</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, papa, maman, maîtresse</t>
+          <t>Amir, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir souffle la poudre de marelle, puis ferme son feutre vert à l'école. Un chuchotement serre son ventre. Le soir, il raconte, et la feuille jaune reste sous le platane.</t>
+          <t>La craie d'hier poudre le pas de la porte. Sur la pierre, un éclat de craie brille. Amir veut la garder, maintenant. Il la saisit trop vite : elle casse, la poudre pique. À l'école, une voix parle d'un secret. Il veut le dire tout de suite : les mots se perdent. Il refuse de foncer, raconte le soir. Merci vécu. Sur la pierre, l'éclat de craie tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>De la craie blanche poudre le pas de la porte. Un platane du village bouge, tout lent. Une feuille tourne, puis s'arrête. Papa secoue le tapis. Un nuage gris s'envole. Maman ferme la boîte des feutres, clic. Ça sent le bois du tapis et l'air du matin. Il reste de la marelle, d'hier. La craie a fait un petit chemin blanc. En ce moment, Amir souffle sur la craie. La poudre vole, puis retombe. Elle pique le nez, papa. Souffle à côté. Amir souffle sur le côté. La poudre part vers le platane. Tes pieds restent sur la pierre. Je veux emporter le feutre vert. Pour la marelle, plus tard. Tu as tes feutres dans la boîte ? Oui, maman. Clic. Le platane a encore des feuilles jaunes, tu vois ? Oui. Une est tombée. On la laisse. Elle est jolie par terre. On y va. Tu dis au revoir à maman. Au revoir, maman. Je t'écoute ce soir, Amir. L'école sent les feutres et le papier. Bonjour. On range les feutres. Bonjour, maîtresse. Amir écoute. Il range son feutre vert, le bouchon bien fermé. Le vert sent un peu fort, tout près. Merci, Amir. Plus tard, quelqu'un s'approche. Une voix parle tout bas, d'un secret. Amir sent un malaise. Son ventre se serre. Il repose les mains sur ses genoux. Il reste près de sa chaise. Le soir, la craie est encore sur la pierre. La porte s'ouvre. Te voilà. Le tapis est rentré. Amir regarde le chemin blanc. La feuille jaune est encore là. Le ventre est encore serré.</t>
+          <t>La craie d'hier poudre le pas de la porte. Le platane du village bouge ses branches. Une feuille jaune tourne, puis s'arrête. Papa secoue le tapis. Un nuage gris s'envole. Maman ferme la boîte des feutres, clic. Ça sent le bois du tapis et l'air du matin. Il reste de la marelle, d'hier. La craie a fait un petit chemin blanc. Sur la pierre, un éclat de craie brille. Il est petit, papa. C'est la craie d'hier. Je la prends, maintenant ! En ce moment, Amir saisit la craie. La craie casse entre ses doigts. La poudre vole, puis retombe. Elle pique le nez, papa ! L'éclat de craie tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas ! Tu souffles à côté ? Papa s'accroupit à la même hauteur. Amir souffle trop fort, trop vite. La poudre lui revient au visage. Oh. Ses épaules tombent un peu. Tes pieds sont sur la pierre ? Oui, papa. Tes feutres sont dans la boîte ? Oui, maman. Clic. Tu vois la feuille jaune ? Oui. Elle est tombée. On la laisse par terre ? Oui, elle est jolie. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le chemin sent la pierre froide. Une feuille jaune tape le platane. L'école sent les feutres et le papier. La maîtresse parle près du tableau. Bonjour. Bonjour, maîtresse. Amir pose le feutre vert, bouchon fermé. Le vert sent un peu fort, tout près. Une poussière de tableau flotte dans l'air. Plus tard, une voix s'approche. Elle parle bas, d'un secret. Amir sent un malaise. Son ventre se serre. Je le dis, maintenant ! Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Amir referme la bouche. Il repose les mains sur ses genoux. Il reste près de sa chaise. Le soir, la porte s'ouvre. Ça sent le tapis et la pierre. Te voilà, Amir. Le tapis est rentré. La craie attend sur la pierre. La feuille jaune est là. Le ventre est serré, tout petit. Amir regarde papa. Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>De la craie blanche poudre le pas de la porte. Un platane du village bouge, tout lent. Une feuille tourne, puis s'arrête. Papa secoue le tapis. Un nuage gris s'envole. Maman ferme la boîte des feutres, clic. Ça sent le bois du tapis et l'air du matin. Il reste de la marelle, d'hier. La craie a fait un petit chemin blanc. En ce moment, Amir souffle sur la craie. La poudre vole, puis retombe. Elle pique le nez, papa. Souffle à côté. Amir souffle sur le côté. La poudre part vers le platane. Tes pieds restent sur la pierre. Je veux emporter le feutre vert. Pour la marelle, plus tard. Tu as tes feutres dans la boîte ? Oui, maman. Clic. Le platane a encore des feuilles jaunes, tu vois ? Oui. Une est tombée. On la laisse. Elle est jolie par terre. On y va. Tu dis au revoir à maman. Au revoir, maman. Je t'écoute ce soir, Amir. L'école sent les feutres et le papier. Bonjour. On range les feutres. Bonjour, maîtresse. Amir écoute. Il range son feutre vert, le bouchon bien fermé. Le vert sent un peu fort, tout près. Merci, Amir. Plus tard, quelqu'un s'approche. Une voix parle tout bas, d'un secret. Amir sent un malaise. Son ventre se serre. Il repose les mains sur ses genoux. Il reste près de sa chaise. Le soir, la craie est encore sur la pierre. La porte s'ouvre. Te voilà. Le tapis est rentré. Amir regarde le chemin blanc. La feuille jaune est encore là. Le ventre est encore serré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La craie d'hier poudre le pas de la porte. Le platane du village bouge ses branches. Une feuille jaune tourne, puis s'arrête. Papa secoue le tapis. Un nuage gris s'envole. Maman ferme la boîte des feutres, clic. Ça sent le bois du tapis et l'air du matin. Il reste de la marelle, d'hier. La craie a fait un petit chemin blanc. Sur la pierre, un &lt;emphasis level="moderate"&gt;éclat de craie&lt;/emphasis&gt; brille. Il est petit, papa. C'est la craie d'hier. Je la prends, maintenant ! En ce moment, Amir saisit la craie. La craie casse entre ses doigts. La poudre vole, puis retombe. Elle pique le nez, papa ! L'éclat de craie tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas ! Tu souffles à côté ? Papa s'accroupit à la même hauteur. Amir souffle trop fort, trop vite. La poudre lui revient au visage. Oh. Ses épaules tombent un peu. Tes pieds sont sur la pierre ? Oui, papa. Tes feutres sont dans la boîte ? Oui, maman. Clic. Tu vois la feuille jaune ? Oui. Elle est tombée. On la laisse par terre ? Oui, elle est jolie. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le chemin sent la pierre froide. Une feuille jaune tape le platane. L'école sent les feutres et le papier. La maîtresse parle près du tableau. Bonjour. Bonjour, maîtresse. Amir pose le feutre vert, bouchon fermé. Le vert sent un peu fort, tout près. Une poussière de tableau flotte dans l'air. Plus tard, une voix s'approche. Elle parle bas, d'un secret. Amir sent un malaise. Son ventre se serre. Je le dis, maintenant ! Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Amir referme la bouche. Il repose les mains sur ses genoux. Il reste près de sa chaise. Le soir, la porte s'ouvre. Ça sent le tapis et la pierre. Te voilà, Amir. Le tapis est rentré. La craie attend sur la pierre. La feuille jaune est là. Le ventre est serré, tout petit. Amir regarde papa. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ninon est à l'école. La maîtresse parle. Ninon aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les feutres. Ninon range son feutre. Elle écoute bien. Plus tard, un camarade chuchote. Il dit : c'est un secret. Garde ça pour toi. Ninon sent un malaise. Son ventre est serré. Le soir, papa l'attend. Ninon vient raconter à la maison. Elle dit : papa, j'ai eu un malaise. Un camarade a parlé d'un secret. Papa l'écoute. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman. [pause]</t>
+          <t>La craie d'hier poudre le pas de la porte. Le platane du village bouge ses branches. Une feuille jaune tourne, puis s'arrête. Papa secoue le tapis. Un nuage gris s'envole. Maman ferme la boîte des feutres, clic. Ça sent le bois du tapis et l'air du matin. Il reste de la marelle, d'hier. La craie a fait un petit chemin blanc. Sur la pierre, un &lt;emphasis&gt;éclat de craie&lt;/emphasis&gt; brille. Il est petit, papa. C'est la craie d'hier. Je la prends, maintenant ! En ce moment, Amir saisit la craie. La craie casse entre ses doigts. La poudre vole, puis retombe. Elle pique le nez, papa ! L'éclat de craie tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas ! Tu souffles à côté ? Papa s'accroupit à la même hauteur. Amir souffle trop fort, trop vite. La poudre lui revient au visage. Oh. Ses épaules tombent un peu. Tes pieds sont sur la pierre ? Oui, papa. Tes feutres sont dans la boîte ? Oui, maman. Clic. Tu vois la feuille jaune ? Oui. Elle est tombée. On la laisse par terre ? Oui, elle est jolie. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le chemin sent la pierre froide. Une feuille jaune tape le platane. L'école sent les feutres et le papier. La maîtresse parle près du tableau. Bonjour. Bonjour, maîtresse. Amir pose le feutre vert, bouchon fermé. Le vert sent un peu fort, tout près. Une poussière de tableau flotte dans l'air. Plus tard, une voix s'approche. Elle parle bas, d'un secret. Amir sent un malaise. Son ventre se serre. Je le dis, maintenant ! Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Amir referme la bouche. Il repose les mains sur ses genoux. Il reste près de sa chaise. Le soir, la porte s'ouvre. Ça sent le tapis et la pierre. Te voilà, Amir. Le tapis est rentré. La craie attend sur la pierre. La feuille jaune est là. Le ventre est serré, tout petit. Amir regarde papa. Il ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de craie</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,65 +1321,87 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis malaise; intensite=2; destinataire=enfant; sous_texte=il_veut_la_craie_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|De la craie blanche poudre le pas de la porte.
-narrateur|Un platane du village bouge, tout lent.
-narrateur|Une feuille tourne, puis s'arrête.
+          <t>narrateur|La craie d'hier poudre le pas de la porte.
+narrateur|Le platane du village bouge ses branches.
+narrateur|Une feuille jaune tourne, puis s'arrête.
 narrateur|Papa secoue le tapis.
 narrateur|Un nuage gris s'envole.
 narrateur|Maman ferme la boîte des feutres, clic.
 narrateur|Ça sent le bois du tapis et l'air du matin.
 papa|Il reste de la marelle, d'hier.
 maman|La craie a fait un petit chemin blanc.
-narrateur|En ce moment, Amir souffle sur la craie.
+narrateur|Sur la pierre, un éclat de craie brille.
+enfant-m|Il est petit, papa.
+papa|C'est la craie d'hier.
+enfant-m|Je la prends, maintenant !
+narrateur|En ce moment, Amir saisit la craie.
+narrateur|La craie casse entre ses doigts.
 narrateur|La poudre vole, puis retombe.
-enfant-m|Elle pique le nez, papa.
-papa|Souffle à côté.
-narrateur|Amir souffle sur le côté.
-narrateur|La poudre part vers le platane.
-papa|Tes pieds restent sur la pierre.
-enfant-m|Je veux emporter le feutre vert.
-enfant-m|Pour la marelle, plus tard.
-maman|Tu as tes feutres dans la boîte ?
+enfant-m|Elle pique le nez, papa !
+narrateur|L'éclat de craie tremble, puis tient.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Ça ne veut pas !
+papa|Tu souffles à côté ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Amir souffle trop fort, trop vite.
+narrateur|La poudre lui revient au visage.
+enfant-m|Oh.
+narrateur|Ses épaules tombent un peu.
+papa|Tes pieds sont sur la pierre ?
+enfant-m|Oui, papa.
+maman|Tes feutres sont dans la boîte ?
 enfant-m|Oui, maman.
 enfant-m|Clic.
-papa|Le platane a encore des feuilles jaunes, tu vois ?
+papa|Tu vois la feuille jaune ?
 enfant-m|Oui.
-enfant-m|Une est tombée.
-maman|On la laisse.
-maman|Elle est jolie par terre.
-papa|On y va.
-papa|Tu dis au revoir à maman.
+enfant-m|Elle est tombée.
+maman|On la laisse par terre ?
+enfant-m|Oui, elle est jolie.
+papa|On y va ?
+enfant-m|On y va.
 enfant-m|Au revoir, maman.
-maman|Je t'écoute ce soir, Amir.
+maman|Au revoir, Amir.
+narrateur|Dehors, le chemin sent la pierre froide.
+narrateur|Une feuille jaune tape le platane.
 narrateur|L'école sent les feutres et le papier.
+narrateur|La maîtresse parle près du tableau.
 maitresse|Bonjour.
-maitresse|On range les feutres.
 enfant-m|Bonjour, maîtresse.
-narrateur|Amir écoute.
-narrateur|Il range son feutre vert, le bouchon bien fermé.
+narrateur|Amir pose le feutre vert, bouchon fermé.
 narrateur|Le vert sent un peu fort, tout près.
-maitresse|Merci, Amir.
-narrateur|Plus tard, quelqu'un s'approche.
-narrateur|Une voix parle tout bas, d'un secret.
+narrateur|Une poussière de tableau flotte dans l'air.
+narrateur|Plus tard, une voix s'approche.
+narrateur|Elle parle bas, d'un secret.
 narrateur|Amir sent un malaise.
 narrateur|Son ventre se serre.
+enfant-m|Je le dis, maintenant !
+narrateur|Ses mots se cognent à ceux de la classe.
+narrateur|Personne ne tourne la tête.
+narrateur|Amir referme la bouche.
 narrateur|Il repose les mains sur ses genoux.
 narrateur|Il reste près de sa chaise.
-narrateur|Le soir, la craie est encore sur la pierre.
-narrateur|La porte s'ouvre.
-papa|Te voilà.
+narrateur|Le soir, la porte s'ouvre.
+narrateur|Ça sent le tapis et la pierre.
+papa|Te voilà, Amir.
 papa|Le tapis est rentré.
-narrateur|Amir regarde le chemin blanc.
-narrateur|La feuille jaune est encore là.
-narrateur|Le ventre est encore serré.</t>
+narrateur|La craie attend sur la pierre.
+narrateur|La feuille jaune est là.
+narrateur|Le ventre est serré, tout petit.
+narrateur|Amir regarde papa.
+narrateur|Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>porte,pas</t>
+          <t>craie,tapis</t>
         </is>
       </c>
     </row>
@@ -1411,12 +1433,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir a un malaise. Que fait-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ninon a un malaise. Que fait-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1426,7 +1448,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>raconter | il raconte | à papa | à la maison | écouter</t>
+          <t>raconter | il raconte | à papa | à la maison | il dit | le secret | il parle | papa maman</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1441,7 +1463,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il raconte à papa. Que fait Amir ?</t>
+          <t>Amir a un malaise à la maison. Que fait-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1479,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1490,7 +1512,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1505,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1547,17 +1573,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_raconte_a_la_maison; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1590,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Papa. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Viens sur la pierre, près de nous. Amir parle. Papa écoute. Maman écoute. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. Le ventre d'Amir se desserre.</t>
+          <t>Amir ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. Le tapis est sec, Amir. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il pose les mains à plat. Le pas de la porte est calme. Tes pieds sont sur la pierre ? Papa pose le tapis contre le mur. La feuille jaune est sous le platane. Maman n'a pas fini non plus. Amir attend que le silence arrive. Sur la pierre, l'éclat de craie brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Une voix a parlé d'un secret. Mon ventre s'est serré. Merci, Amir. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Amir pose la main sur la pierre froide. Le ventre d'Amir se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Papa. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Viens sur la pierre, près de nous. Amir parle. Papa écoute. Maman écoute. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. Le ventre d'Amir se desserre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir ouvre la bouche trop vite. Papa, un &lt;emphasis level="moderate"&gt;secret&lt;/emphasis&gt;. Papa n'a pas fini sa phrase. Le tapis est sec, Amir. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il pose les mains à plat. Le pas de la porte est calme. Tes pieds sont sur la pierre ? Papa pose le tapis contre le mur. La feuille jaune est sous le platane. Maman n'a pas fini non plus. Amir attend que le silence arrive. Sur la pierre, l'éclat de craie brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Une voix a parlé d'un secret. Mon ventre s'est serré. Merci, Amir. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Amir pose la main sur la pierre froide. Le ventre d'Amir se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ninon a écouté la maîtresse. Elle a raconté son malaise à la maison. Papa est là. [pause]</t>
+          <t>Amir ouvre la bouche trop vite. Papa, un &lt;emphasis&gt;secret&lt;/emphasis&gt;. Papa n'a pas fini sa phrase. Le tapis est sec, Amir. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il pose les mains à plat. Le pas de la porte est calme. Tes pieds sont sur la pierre ? Papa pose le tapis contre le mur. La feuille jaune est sous le platane. Maman n'a pas fini non plus. Amir attend que le silence arrive. Sur la pierre, l'éclat de craie brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Une voix a parlé d'un secret. Mon ventre s'est serré. Merci, Amir. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Amir pose la main sur la pierre froide. Le ventre d'Amir se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1647,7 +1673,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1655,10 +1681,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,28 +1705,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>secret</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1725,23 +1755,44 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_attend_puis_raconte; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Papa.
-enfant-m|J'ai eu un malaise.
-enfant-m|Quelqu'un a parlé d'un secret.
-papa|On t'écoute.
-maman|Viens sur la pierre, près de nous.
-narrateur|Amir parle.
-narrateur|Papa écoute.
-narrateur|Maman écoute.
-papa|Tu as bien fait de raconter.
-maman|À l'école, on écoute la maîtresse.
-papa|Si tu as un malaise, tu viens le dire.
+          <t>narrateur|Amir ouvre la bouche trop vite.
+enfant-m|Papa, un secret.
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le tapis est sec, Amir.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Il pose les mains à plat.
+narrateur|Le pas de la porte est calme.
+papa|Tes pieds sont sur la pierre ?
+narrateur|Papa pose le tapis contre le mur.
+maman|La feuille jaune est sous le platane.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Amir attend que le silence arrive.
+narrateur|Sur la pierre, l'éclat de craie brille.
+enfant-m|Il est là.
+enfant-m|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-m|Une voix a parlé d'un secret.
+enfant-m|Mon ventre s'est serré.
+papa|Merci, Amir.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu veux un peu d'eau ?
+enfant-m|Oui, maman.
+narrateur|Amir pose la main sur la pierre froide.
 narrateur|Le ventre d'Amir se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pierre,voix</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1819,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman verse un peu d'eau dans un verre. L'eau fait un petit bruit clair. Tu veux un peu d'eau ? Oui. Merci, maman. Amir boit une gorgée. Tu as tes pieds sur la pierre ? Oui, papa. Amir souffle encore, à côté de la craie. Un peu de poudre s'envole. Elle ne pique plus. La feuille jaune est toujours là. On la laisse. On reste encore un peu ensemble ? Oui, papa. Le platane bouge, tout lent.</t>
+          <t>Maman verse de l'eau dans un verre. L'eau fait un petit bruit clair. C'est froid. Tes pieds sont au chaud ? Oui, sur la pierre. Amir boit une gorgée. Amir veut souffler la craie, tout de suite. Il souffle trop fort. La poudre lui pique les yeux. Oh. Amir s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il écoute le platane, un instant. Il souffle à côté, plus léger. Un peu de poudre s'envole vers l'arbre. Elle ne pique plus. On laisse la feuille jaune ? Oui, par terre. On reste un peu ? Oui, papa. Le platane bouge ses branches.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman verse un peu d'eau dans un verre. L'eau fait un petit bruit clair. Tu veux un peu d'eau ? Oui. Merci, maman. Amir boit une gorgée. Tu as tes pieds sur la pierre ? Oui, papa. Amir souffle encore, à côté de la craie. Un peu de poudre s'envole. Elle ne pique plus. La feuille jaune est toujours là. On la laisse. On reste encore un peu ensemble ? Oui, papa. Le platane bouge, tout lent.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman verse de l'eau dans un verre. L'eau fait un petit bruit clair. C'est froid. Tes pieds sont au chaud ? Oui, sur la pierre. Amir boit une gorgée. Amir veut souffler la craie, tout de suite. Il souffle trop fort. La &lt;emphasis level="moderate"&gt;poudre&lt;/emphasis&gt; lui pique les yeux. Oh. Amir s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il écoute le platane, un instant. Il souffle à côté, plus léger. Un peu de poudre s'envole vers l'arbre. Elle ne pique plus. On laisse la feuille jaune ? Oui, par terre. On reste un peu ? Oui, papa. Le platane bouge ses branches.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ninon boit un verre d'eau. Papa lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Maman verse de l'eau dans un verre. L'eau fait un petit bruit clair. C'est froid. Tes pieds sont au chaud ? Oui, sur la pierre. Amir boit une gorgée. Amir veut souffler la craie, tout de suite. Il souffle trop fort. La &lt;emphasis&gt;poudre&lt;/emphasis&gt; lui pique les yeux. Oh. Amir s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il écoute le platane, un instant. Il souffle à côté, plus léger. Un peu de poudre s'envole vers l'arbre. Elle ne pique plus. On laisse la feuille jaune ? Oui, par terre. On reste un peu ? Oui, papa. Le platane bouge ses branches. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1825,7 +1876,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1833,10 +1884,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1859,30 +1910,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>poudre</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1891,10 +1942,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1905,25 +1956,40 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_souffler_trop_fort; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman verse un peu d'eau dans un verre.
+          <t>narrateur|Maman verse de l'eau dans un verre.
 narrateur|L'eau fait un petit bruit clair.
-maman|Tu veux un peu d'eau ?
-enfant-m|Oui.
-enfant-m|Merci, maman.
+enfant-m|C'est froid.
+papa|Tes pieds sont au chaud ?
+enfant-m|Oui, sur la pierre.
 narrateur|Amir boit une gorgée.
-papa|Tu as tes pieds sur la pierre ?
+narrateur|Amir veut souffler la craie, tout de suite.
+narrateur|Il souffle trop fort.
+narrateur|La poudre lui pique les yeux.
+enfant-m|Oh.
+narrateur|Amir s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il refuse de foncer.
+narrateur|Il écoute le platane, un instant.
+narrateur|Il souffle à côté, plus léger.
+narrateur|Un peu de poudre s'envole vers l'arbre.
+enfant-m|Elle ne pique plus.
+maman|On laisse la feuille jaune ?
+enfant-m|Oui, par terre.
+papa|On reste un peu ?
 enfant-m|Oui, papa.
-narrateur|Amir souffle encore, à côté de la craie.
-narrateur|Un peu de poudre s'envole.
-enfant-m|Elle ne pique plus.
-maman|La feuille jaune est toujours là.
-enfant-m|On la laisse.
-papa|On reste encore un peu ensemble ?
-enfant-m|Oui, papa.
-narrateur|Le platane bouge, tout lent.</t>
+narrateur|Le platane bouge ses branches.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>eau,poudre</t>
         </is>
       </c>
     </row>
@@ -1950,17 +2016,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le chemin de craie s'efface un peu. La feuille jaune reste sous le platane. On t'a écouté, Amir. Tu as rangé ton feutre, puis tu as raconté.</t>
+          <t>Ils restent sur le pas de la porte. La poudre blanche repose sur la pierre. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la pierre. On est bien, ici. Le tapis sent le bois, un peu. Amir glisse le pied, sans se presser. La craie repose contre la pierre. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. Le platane repose contre le ciel. Une feuille jaune ne bouge plus. Elle est jolie par terre. On la laisse ? Oui. L'éclat de craie tient sur la pierre.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le chemin de craie s'efface un peu. La feuille jaune reste sous le platane. On t'a écouté, Amir. Tu as rangé ton feutre, puis tu as raconté.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent sur le pas de la porte. La poudre blanche repose sur la pierre. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la pierre. On est bien, ici. Le tapis sent le bois, un peu. Amir glisse le pied, sans se presser. La craie repose contre la pierre. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. Le platane repose contre le ciel. Une feuille jaune ne bouge plus. Elle est jolie par terre. On la laisse ? Oui. L'&lt;emphasis level="moderate"&gt;éclat de craie&lt;/emphasis&gt; tient sur la pierre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent sur le pas de la porte. La poudre blanche repose sur la pierre. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la pierre. On est bien, ici. Le tapis sent le bois, un peu. Amir glisse le pied, sans se presser. La craie repose contre la pierre. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. Le platane repose contre le ciel. Une feuille jaune ne bouge plus. Elle est jolie par terre. On la laisse ? Oui. L'&lt;emphasis&gt;éclat de craie&lt;/emphasis&gt; tient sur la pierre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,7 +2073,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2015,10 +2081,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2027,12 +2093,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2107,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de craie</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2130,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,27 +2143,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_pierre; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le chemin de craie s'efface un peu.
-narrateur|La feuille jaune reste sous le platane.
-papa|On t'a écouté, Amir.
-maman|Tu as rangé ton feutre, puis tu as raconté.</t>
+          <t>narrateur|Ils restent sur le pas de la porte.
+narrateur|La poudre blanche repose sur la pierre.
+enfant-m|Comme ce matin, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur la pierre.
+maman|On est bien, ici.
+narrateur|Le tapis sent le bois, un peu.
+narrateur|Amir glisse le pied, sans se presser.
+narrateur|La craie repose contre la pierre.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes joues ?
+enfant-m|Oui, il est frais.
+narrateur|Le platane repose contre le ciel.
+narrateur|Une feuille jaune ne bouge plus.
+enfant-m|Elle est jolie par terre.
+papa|On la laisse ?
+enfant-m|Oui.
+narrateur|L'éclat de craie tient sur la pierre.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>platane,pierre</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2206,6 +2299,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>